<commit_message>
NEW RELEASE WITH TRACK PANT AND COUTNER UI AND NEW BATCH BUTTON
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="74">
   <si>
     <t>kind</t>
   </si>
@@ -97,7 +97,7 @@
     <t>BEIGE</t>
   </si>
   <si>
-    <t>F-34-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-34-Beige-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Active</t>
@@ -121,16 +121,16 @@
     <t>Made In India</t>
   </si>
   <si>
-    <t>F-32-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-32-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-Beige-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Inactive</t>
@@ -139,19 +139,19 @@
     <t>ICE</t>
   </si>
   <si>
-    <t>F-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Shorts</t>
@@ -160,34 +160,34 @@
     <t>XL</t>
   </si>
   <si>
-    <t>F-Shorts-XL-Black-01-</t>
+    <t>FB-Shorts-XL-Black-01-</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>F-Shorts-L-Black-01-</t>
+    <t>FB-Shorts-L-Black-01-</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>F-Shorts-M-Black-01-</t>
+    <t>FB-Shorts-M-Black-01-</t>
   </si>
   <si>
     <t>Trouser</t>
   </si>
   <si>
-    <t>F-M-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-L-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-XL-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-S-TROUSER-BLACk-01-</t>
+    <t>FB-M-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-L-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-XL-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-S-TROUSER-BLACk-01-</t>
   </si>
   <si>
     <t>S</t>
@@ -196,22 +196,34 @@
     <t>Black-baggy</t>
   </si>
   <si>
-    <t>F-34-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-32-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>How to use</t>
+    <t>FB-34-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>Track Pant</t>
+  </si>
+  <si>
+    <t>FB-M-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-L-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-XL-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-S-TRACK-PANT-BLACk-01-</t>
   </si>
   <si>
     <t>Use one row per product/size combination.</t>
@@ -597,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA34"/>
+  <dimension ref="A1:AA42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42.142857142857146" customWidth="1"/>
@@ -716,7 +728,7 @@
         <v>29</v>
       </c>
       <c r="E2">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F2">
         <v>459</v>
@@ -796,7 +808,7 @@
         <v>29</v>
       </c>
       <c r="E3">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F3">
         <v>459</v>
@@ -876,7 +888,7 @@
         <v>29</v>
       </c>
       <c r="E4">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F4">
         <v>459</v>
@@ -956,7 +968,7 @@
         <v>29</v>
       </c>
       <c r="E5">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F5">
         <v>459</v>
@@ -1036,7 +1048,7 @@
         <v>40</v>
       </c>
       <c r="E6">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F6">
         <v>459</v>
@@ -1116,7 +1128,7 @@
         <v>29</v>
       </c>
       <c r="E7">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F7">
         <v>469</v>
@@ -1196,7 +1208,7 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F8">
         <v>469</v>
@@ -1276,7 +1288,7 @@
         <v>29</v>
       </c>
       <c r="E9">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F9">
         <v>469</v>
@@ -1356,7 +1368,7 @@
         <v>29</v>
       </c>
       <c r="E10">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F10">
         <v>469</v>
@@ -1436,7 +1448,7 @@
         <v>40</v>
       </c>
       <c r="E11">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F11">
         <v>469</v>
@@ -2396,7 +2408,7 @@
         <v>29</v>
       </c>
       <c r="E23">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F23">
         <v>429</v>
@@ -2476,7 +2488,7 @@
         <v>29</v>
       </c>
       <c r="E24">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F24">
         <v>429</v>
@@ -2556,7 +2568,7 @@
         <v>29</v>
       </c>
       <c r="E25">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F25">
         <v>429</v>
@@ -2636,7 +2648,7 @@
         <v>29</v>
       </c>
       <c r="E26">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F26">
         <v>429</v>
@@ -2716,7 +2728,7 @@
         <v>40</v>
       </c>
       <c r="E27">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F27">
         <v>429</v>
@@ -2782,24 +2794,339 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28">
+        <v>999</v>
+      </c>
+      <c r="F28">
+        <v>315</v>
+      </c>
+      <c r="G28">
+        <v>279</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28" t="s">
+        <v>30</v>
+      </c>
+      <c r="J28" t="s">
+        <v>31</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>250</v>
+      </c>
+      <c r="M28" t="s">
+        <v>32</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28">
+        <v>35</v>
+      </c>
+      <c r="R28">
+        <v>27</v>
+      </c>
+      <c r="S28">
+        <v>2</v>
+      </c>
+      <c r="T28">
+        <v>0.25</v>
+      </c>
+      <c r="U28">
+        <v>6109</v>
+      </c>
+      <c r="W28" t="s">
+        <v>33</v>
+      </c>
+      <c r="X28" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29">
+        <v>999</v>
+      </c>
+      <c r="F29">
+        <v>315</v>
+      </c>
+      <c r="G29">
+        <v>279</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>30</v>
+      </c>
+      <c r="J29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K29">
+        <v>1</v>
+      </c>
+      <c r="L29">
+        <v>250</v>
+      </c>
+      <c r="M29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <v>35</v>
+      </c>
+      <c r="R29">
+        <v>27</v>
+      </c>
+      <c r="S29">
+        <v>2</v>
+      </c>
+      <c r="T29">
+        <v>0.25</v>
+      </c>
+      <c r="U29">
+        <v>6109</v>
+      </c>
+      <c r="W29" t="s">
+        <v>33</v>
+      </c>
+      <c r="X29" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z29" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30">
+        <v>999</v>
+      </c>
+      <c r="F30">
+        <v>315</v>
+      </c>
+      <c r="G30">
+        <v>279</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" t="s">
+        <v>31</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30">
+        <v>250</v>
+      </c>
+      <c r="M30" t="s">
+        <v>32</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30">
+        <v>35</v>
+      </c>
+      <c r="R30">
+        <v>27</v>
+      </c>
+      <c r="S30">
+        <v>2</v>
+      </c>
+      <c r="T30">
+        <v>0.25</v>
+      </c>
+      <c r="U30">
+        <v>6109</v>
+      </c>
+      <c r="W30" t="s">
+        <v>33</v>
+      </c>
+      <c r="X30" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z30" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>69</v>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31">
+        <v>999</v>
+      </c>
+      <c r="F31">
+        <v>315</v>
+      </c>
+      <c r="G31">
+        <v>279</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>31</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>250</v>
+      </c>
+      <c r="M31" t="s">
+        <v>32</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31">
+        <v>35</v>
+      </c>
+      <c r="R31">
+        <v>27</v>
+      </c>
+      <c r="S31">
+        <v>2</v>
+      </c>
+      <c r="T31">
+        <v>0.25</v>
+      </c>
+      <c r="U31">
+        <v>6109</v>
+      </c>
+      <c r="W31" t="s">
+        <v>33</v>
+      </c>
+      <c r="X31" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>